<commit_message>
Halves regressions with fye1 fixed effects; fix Panel B note in the split table
First-vs-second-half tables rerun with fiscal-year-end date fixed effects in
place of year effects (plan-FE-only columns dropped), updated benchmark.
The year-FE workbook is regenerated with its split-table note corrected to
describe the updated benchmark (numbers unchanged).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qpw2BayLmQibPr7ZExRA1m
</commit_message>
<xml_diff>
--- a/referee_response/time_to_departure/halves_updated_benchmark.xlsx
+++ b/referee_response/time_to_departure/halves_updated_benchmark.xlsx
@@ -31,7 +31,7 @@
     <t xml:space="preserve">Table XI: Conflicted CIOs: Plan Performance in the First versus Second Half of Tenure (updated benchmark)</t>
   </si>
   <si>
-    <t xml:space="preserve">This table repeats the regressions of Table III, splitting the Conflicted CIO indicator into two indicators: Conflicted CIO x First Half of Tenure, equal to 1 in the fiscal years in which a conflicted CIO's tenure is at most one half of the CIO's tenure at departure, and Conflicted CIO x Second Half of Tenure, equal to 1 in the remaining fiscal years of a conflicted CIO's tenure. The omitted category is all plan-years run by non-conflicted CIOs, so each coefficient is the performance differential of conflicted CIOs in that part of their tenure relative to non-conflicted CIOs. Tenure at departure is the CIO's tenure in the last fiscal year observed in the plan plus any gap to the departure year. 11 conflicted plan-years for which tenure at departure cannot be determined are absorbed by a separate indicator that is not reported. The performance measure in Panel A is Peer-Adjusted Return, which is the difference of a plan's return and the average pension plan return each year. The performance measure in Panel B is Benchmark-Adjusted Return, which is calculated as the plan's return minus the return of its policy benchmark, when available. The other independent variables are as defined in Table I. The last row reports the p-value of a test that the first-half and second-half coefficients are equal. The standard errors are double clustered by plan and year. Coefficients marked with ***, **, and * are significant at the 1%, 5%, and 10% level, respectively.</t>
+    <t xml:space="preserve">This table repeats the regressions of Table III, splitting the Conflicted CIO indicator into two indicators: Conflicted CIO x First Half of Tenure, equal to 1 in the fiscal years in which a conflicted CIO's tenure is at most one half of the CIO's tenure at departure, and Conflicted CIO x Second Half of Tenure, equal to 1 in the remaining fiscal years of a conflicted CIO's tenure. The omitted category is all plan-years run by non-conflicted CIOs, so each coefficient is the performance differential of conflicted CIOs in that part of their tenure relative to non-conflicted CIOs. Tenure at departure is the CIO's tenure in the last fiscal year observed in the plan plus any gap to the departure year. 11 conflicted plan-years for which tenure at departure cannot be determined are absorbed by a separate indicator that is not reported. The performance measure in Panel A is Peer-Adjusted Return, which is the difference of a plan's return and the average pension plan return each year. The performance measure in Panel B is Benchmark-Adjusted Return, which is calculated as the plan's return minus the return of its updated policy benchmark (the benchmark return reported in the plan's financial report or, where none is stated, an inferred value graded A or B). The other independent variables are as defined in Table I. The last row reports the p-value of a test that the first-half and second-half coefficients are equal. The standard errors are double clustered by plan and year. Coefficients marked with ***, **, and * are significant at the 1%, 5%, and 10% level, respectively.</t>
   </si>
   <si>
     <t xml:space="preserve">Panel A. Peer-Adjusted Returns</t>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="270" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E49" s="10" t="n">
         <f aca="false">'Estimates-split'!N29</f>
-        <v>0.0952588261959438</v>
+        <v>0.095258826195944</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="E52" s="13" t="n">
         <f aca="false">'Estimates-split'!Q24</f>
-        <v>0.241981682651842</v>
+        <v>0.241981697416763</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="E99" s="10" t="n">
         <f aca="false">'Estimates-split'!AD29</f>
-        <v>0.12390479939966</v>
+        <v>0.123904799399671</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="E102" s="13" t="n">
         <f aca="false">'Estimates-split'!AG24</f>
-        <v>0.0956110552579578</v>
+        <v>0.0956110118151261</v>
       </c>
     </row>
   </sheetData>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="E48" s="10" t="n">
         <f aca="false">'Estimates-split'!AT29</f>
-        <v>0.670564522582896</v>
+        <v>0.67056452258284</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="E51" s="13" t="n">
         <f aca="false">'Estimates-split'!AW24</f>
-        <v>0.821651149356285</v>
+        <v>0.821651147963641</v>
       </c>
     </row>
   </sheetData>
@@ -7346,18 +7346,18 @@
         <v>0.0340963014993949</v>
       </c>
       <c r="N4" s="26" t="n">
-        <v>-0.860866775829736</v>
+        <v>-0.860866775829676</v>
       </c>
       <c r="O4" s="26" t="n">
-        <v>0.350886983744449</v>
+        <v>0.350886914766573</v>
       </c>
       <c r="P4" s="27" t="n">
         <f aca="false">IF(O4&gt;0,N4/O4,"")</f>
-        <v>-2.45340185219496</v>
+        <v>-2.45340233448821</v>
       </c>
       <c r="Q4" s="27" t="n">
         <f aca="false">IF(O4&gt;0,TDIST(ABS(P4),MIN(N27,N28)-1,2),"")</f>
-        <v>0.024570143932302</v>
+        <v>0.0245701194412032</v>
       </c>
       <c r="R4" s="26" t="n">
         <v>-0.486153585661349</v>
@@ -7402,18 +7402,18 @@
         <v>0.0218057871026355</v>
       </c>
       <c r="AD4" s="26" t="n">
-        <v>-0.684344614208351</v>
+        <v>-0.684344614207798</v>
       </c>
       <c r="AE4" s="26" t="n">
-        <v>0.239277645782293</v>
+        <v>0.239277652502275</v>
       </c>
       <c r="AF4" s="27" t="n">
         <f aca="false">IF(AE4&gt;0,AD4/AE4,"")</f>
-        <v>-2.86004407963376</v>
+        <v>-2.86004399930868</v>
       </c>
       <c r="AG4" s="27" t="n">
         <f aca="false">IF(AE4&gt;0,TDIST(ABS(AF4),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.0104043640408069</v>
+        <v>0.010404365840353</v>
       </c>
       <c r="AH4" s="26" t="n">
         <v>-0.0446206736781622</v>
@@ -7458,18 +7458,18 @@
         <v>0.483811586015004</v>
       </c>
       <c r="AT4" s="26" t="n">
-        <v>0.0365650469337392</v>
+        <v>0.0365650469341304</v>
       </c>
       <c r="AU4" s="26" t="n">
-        <v>0.0546466689479553</v>
+        <v>0.0546466704831331</v>
       </c>
       <c r="AV4" s="27" t="n">
         <f aca="false">IF(AU4&gt;0,AT4/AU4,"")</f>
-        <v>0.669117580955635</v>
+        <v>0.669117562165409</v>
       </c>
       <c r="AW4" s="27" t="n">
         <f aca="false">IF(AU4&gt;0,TDIST(ABS(AV4),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.511912071168239</v>
+        <v>0.51191208287608</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7519,18 +7519,18 @@
         <v>0.0822833079933114</v>
       </c>
       <c r="N5" s="26" t="n">
-        <v>-0.578563222047117</v>
+        <v>-0.578563222047021</v>
       </c>
       <c r="O5" s="26" t="n">
-        <v>0.293549217413428</v>
+        <v>0.293549153896962</v>
       </c>
       <c r="P5" s="27" t="n">
         <f aca="false">IF(O5&gt;0,N5/O5,"")</f>
-        <v>-1.9709240826634</v>
+        <v>-1.9709245091202</v>
       </c>
       <c r="Q5" s="27" t="n">
         <f aca="false">IF(O5&gt;0,TDIST(ABS(P5),MIN(N27,N28)-1,2),"")</f>
-        <v>0.0643083299636531</v>
+        <v>0.0643082775349479</v>
       </c>
       <c r="R5" s="26" t="n">
         <v>-0.330264877962039</v>
@@ -7575,18 +7575,18 @@
         <v>0.320195322812398</v>
       </c>
       <c r="AD5" s="26" t="n">
-        <v>-0.247989277540481</v>
+        <v>-0.247989277539512</v>
       </c>
       <c r="AE5" s="26" t="n">
-        <v>0.230571644076279</v>
+        <v>0.230571622876933</v>
       </c>
       <c r="AF5" s="27" t="n">
         <f aca="false">IF(AE5&gt;0,AD5/AE5,"")</f>
-        <v>-1.0755410906401</v>
+        <v>-1.0755411895239</v>
       </c>
       <c r="AG5" s="27" t="n">
         <f aca="false">IF(AE5&gt;0,TDIST(ABS(AF5),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.296338342397212</v>
+        <v>0.296338299338652</v>
       </c>
       <c r="AH5" s="26" t="n">
         <v>-0.0467075485935625</v>
@@ -7631,18 +7631,18 @@
         <v>0.601526059465714</v>
       </c>
       <c r="AT5" s="26" t="n">
-        <v>0.0278937013870986</v>
+        <v>0.0278937013872841</v>
       </c>
       <c r="AU5" s="26" t="n">
-        <v>0.0562932014253682</v>
+        <v>0.0562932033647532</v>
       </c>
       <c r="AV5" s="27" t="n">
         <f aca="false">IF(AU5&gt;0,AT5/AU5,"")</f>
-        <v>0.495507462372328</v>
+        <v>0.495507445304652</v>
       </c>
       <c r="AW5" s="27" t="n">
         <f aca="false">IF(AU5&gt;0,TDIST(ABS(AV5),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.626237023950058</v>
+        <v>0.626237035758388</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7692,18 +7692,18 @@
         <v>0.24856760929225</v>
       </c>
       <c r="N6" s="26" t="n">
-        <v>0.000222697439686628</v>
+        <v>0.000222697439682929</v>
       </c>
       <c r="O6" s="26" t="n">
-        <v>0.0164563850136208</v>
+        <v>0.016456384332229</v>
       </c>
       <c r="P6" s="27" t="n">
         <f aca="false">IF(O6&gt;0,N6/O6,"")</f>
-        <v>0.0135325856500261</v>
+        <v>0.0135325862101304</v>
       </c>
       <c r="Q6" s="27" t="n">
         <f aca="false">IF(O6&gt;0,TDIST(ABS(P6),MIN(N27,N28)-1,2),"")</f>
-        <v>0.989351753947724</v>
+        <v>0.989351753507062</v>
       </c>
       <c r="R6" s="26" t="n">
         <v>-0.00314810803893259</v>
@@ -7748,18 +7748,18 @@
         <v>0.739592583781502</v>
       </c>
       <c r="AD6" s="26" t="n">
-        <v>-0.0170244542820252</v>
+        <v>-0.017024454282035</v>
       </c>
       <c r="AE6" s="26" t="n">
-        <v>0.016408916793711</v>
+        <v>0.0164089120162451</v>
       </c>
       <c r="AF6" s="27" t="n">
         <f aca="false">IF(AE6&gt;0,AD6/AE6,"")</f>
-        <v>-1.03751237793771</v>
+        <v>-1.03751268001075</v>
       </c>
       <c r="AG6" s="27" t="n">
         <f aca="false">IF(AE6&gt;0,TDIST(ABS(AF6),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.313234665215388</v>
+        <v>0.313234528319919</v>
       </c>
       <c r="AH6" s="26" t="n">
         <v>-0.000253343378606424</v>
@@ -7804,18 +7804,18 @@
         <v>0.247100222764307</v>
       </c>
       <c r="AT6" s="26" t="n">
-        <v>-0.00121104949019937</v>
+        <v>-0.0012110494901976</v>
       </c>
       <c r="AU6" s="26" t="n">
-        <v>0.00050705158101823</v>
+        <v>0.000507051736669438</v>
       </c>
       <c r="AV6" s="27" t="n">
         <f aca="false">IF(AU6&gt;0,AT6/AU6,"")</f>
-        <v>-2.38841477974966</v>
+        <v>-2.38841404656725</v>
       </c>
       <c r="AW6" s="27" t="n">
         <f aca="false">IF(AU6&gt;0,TDIST(ABS(AV6),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.0280863396166101</v>
+        <v>0.0280863818169021</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7865,18 +7865,18 @@
         <v>0.0234081295935938</v>
       </c>
       <c r="N7" s="26" t="n">
-        <v>-1.4177009706968</v>
+        <v>-1.41770097069614</v>
       </c>
       <c r="O7" s="26" t="n">
-        <v>0.725804348754759</v>
+        <v>0.725804356360736</v>
       </c>
       <c r="P7" s="27" t="n">
         <f aca="false">IF(O7&gt;0,N7/O7,"")</f>
-        <v>-1.95328255214936</v>
+        <v>-1.95328253167927</v>
       </c>
       <c r="Q7" s="27" t="n">
         <f aca="false">IF(O7&gt;0,TDIST(ABS(P7),MIN(N27,N28)-1,2),"")</f>
-        <v>0.0665101879553404</v>
+        <v>0.0665101905488387</v>
       </c>
       <c r="R7" s="26" t="n">
         <v>-0.0503616577768491</v>
@@ -7921,18 +7921,18 @@
         <v>0.0850392317405355</v>
       </c>
       <c r="AD7" s="26" t="n">
-        <v>-0.242169104155013</v>
+        <v>-0.24216910415322</v>
       </c>
       <c r="AE7" s="26" t="n">
-        <v>0.718041403644612</v>
+        <v>0.718041388453026</v>
       </c>
       <c r="AF7" s="27" t="n">
         <f aca="false">IF(AE7&gt;0,AD7/AE7,"")</f>
-        <v>-0.337263426490198</v>
+        <v>-0.337263433623176</v>
       </c>
       <c r="AG7" s="27" t="n">
         <f aca="false">IF(AE7&gt;0,TDIST(ABS(AF7),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.739819211101615</v>
+        <v>0.739819205814821</v>
       </c>
       <c r="AH7" s="26" t="n">
         <v>-0.0222747633408498</v>
@@ -7977,18 +7977,18 @@
         <v>0.877604264986718</v>
       </c>
       <c r="AT7" s="26" t="n">
-        <v>0.042342004668457</v>
+        <v>0.0423420046679082</v>
       </c>
       <c r="AU7" s="26" t="n">
-        <v>0.103036485140785</v>
+        <v>0.103036494501161</v>
       </c>
       <c r="AV7" s="27" t="n">
         <f aca="false">IF(AU7&gt;0,AT7/AU7,"")</f>
-        <v>0.41094185822238</v>
+        <v>0.410941820884941</v>
       </c>
       <c r="AW7" s="27" t="n">
         <f aca="false">IF(AU7&gt;0,TDIST(ABS(AV7),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.685966100080684</v>
+        <v>0.685966126966835</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8038,18 +8038,18 @@
         <v>0.0051922091685381</v>
       </c>
       <c r="N8" s="26" t="n">
-        <v>-0.0303912498402354</v>
+        <v>-0.0303912498402368</v>
       </c>
       <c r="O8" s="26" t="n">
-        <v>0.0103010714999345</v>
+        <v>0.0103010724798028</v>
       </c>
       <c r="P8" s="27" t="n">
         <f aca="false">IF(O8&gt;0,N8/O8,"")</f>
-        <v>-2.95029986350727</v>
+        <v>-2.9502995828662</v>
       </c>
       <c r="Q8" s="27" t="n">
         <f aca="false">IF(O8&gt;0,TDIST(ABS(P8),MIN(N27,N28)-1,2),"")</f>
-        <v>0.00856108338700037</v>
+        <v>0.00856108859456663</v>
       </c>
       <c r="R8" s="26" t="n">
         <v>0.00328356989325237</v>
@@ -8094,18 +8094,18 @@
         <v>0.137926000433435</v>
       </c>
       <c r="AD8" s="26" t="n">
-        <v>-0.0170783672354676</v>
+        <v>-0.0170783672354707</v>
       </c>
       <c r="AE8" s="26" t="n">
-        <v>0.0115002544046696</v>
+        <v>0.011500247622076</v>
       </c>
       <c r="AF8" s="27" t="n">
         <f aca="false">IF(AE8&gt;0,AD8/AE8,"")</f>
-        <v>-1.48504255945269</v>
+        <v>-1.48504343529845</v>
       </c>
       <c r="AG8" s="27" t="n">
         <f aca="false">IF(AE8&gt;0,TDIST(ABS(AF8),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.154835415636876</v>
+        <v>0.154835185759317</v>
       </c>
       <c r="AH8" s="26" t="n">
         <v>-0.000820222187063041</v>
@@ -8150,18 +8150,18 @@
         <v>0.267894511893026</v>
       </c>
       <c r="AT8" s="26" t="n">
-        <v>-0.00235462478691992</v>
+        <v>-0.00235462478691389</v>
       </c>
       <c r="AU8" s="26" t="n">
-        <v>0.000988004261744498</v>
+        <v>0.000988003048461075</v>
       </c>
       <c r="AV8" s="27" t="n">
         <f aca="false">IF(AU8&gt;0,AT8/AU8,"")</f>
-        <v>-2.38321318853667</v>
+        <v>-2.38321611515418</v>
       </c>
       <c r="AW8" s="27" t="n">
         <f aca="false">IF(AU8&gt;0,TDIST(ABS(AV8),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.028387226074299</v>
+        <v>0.0283870559407016</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8211,18 +8211,18 @@
         <v>0.566730997868314</v>
       </c>
       <c r="N9" s="26" t="n">
-        <v>-0.0288654016346286</v>
+        <v>-0.0288654016345769</v>
       </c>
       <c r="O9" s="26" t="n">
-        <v>0.0860405960045373</v>
+        <v>0.086040597559141</v>
       </c>
       <c r="P9" s="27" t="n">
         <f aca="false">IF(O9&gt;0,N9/O9,"")</f>
-        <v>-0.335485840115593</v>
+        <v>-0.335485834053348</v>
       </c>
       <c r="Q9" s="27" t="n">
         <f aca="false">IF(O9&gt;0,TDIST(ABS(P9),MIN(N27,N28)-1,2),"")</f>
-        <v>0.741137129070262</v>
+        <v>0.74113713356627</v>
       </c>
       <c r="R9" s="26" t="n">
         <v>-0.17100282538294</v>
@@ -8267,18 +8267,18 @@
         <v>0.988828157018879</v>
       </c>
       <c r="AD9" s="26" t="n">
-        <v>0.0199293355117399</v>
+        <v>0.0199293355119386</v>
       </c>
       <c r="AE9" s="26" t="n">
-        <v>0.171843752602377</v>
+        <v>0.171843763996169</v>
       </c>
       <c r="AF9" s="27" t="n">
         <f aca="false">IF(AE9&gt;0,AD9/AE9,"")</f>
-        <v>0.115973581872677</v>
+        <v>0.115973574184414</v>
       </c>
       <c r="AG9" s="27" t="n">
         <f aca="false">IF(AE9&gt;0,TDIST(ABS(AF9),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.908957549604427</v>
+        <v>0.90895755561144</v>
       </c>
       <c r="AH9" s="26" t="n">
         <v>-0.0393611173108143</v>
@@ -8323,18 +8323,18 @@
         <v>0.167779046470517</v>
       </c>
       <c r="AT9" s="26" t="n">
-        <v>-0.0859817474768352</v>
+        <v>-0.0859817474769594</v>
       </c>
       <c r="AU9" s="26" t="n">
-        <v>0.0554527565948336</v>
+        <v>0.0554527552189633</v>
       </c>
       <c r="AV9" s="27" t="n">
         <f aca="false">IF(AU9&gt;0,AT9/AU9,"")</f>
-        <v>-1.55054054580302</v>
+        <v>-1.55054058427661</v>
       </c>
       <c r="AW9" s="27" t="n">
         <f aca="false">IF(AU9&gt;0,TDIST(ABS(AV9),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.138415687961424</v>
+        <v>0.138415678760493</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8384,18 +8384,18 @@
         <v>0.547250051504808</v>
       </c>
       <c r="N10" s="26" t="n">
-        <v>-0.035065367277741</v>
+        <v>-0.0350653672776936</v>
       </c>
       <c r="O10" s="26" t="n">
-        <v>0.096834522332305</v>
+        <v>0.0968345346341021</v>
       </c>
       <c r="P10" s="27" t="n">
         <f aca="false">IF(O10&gt;0,N10/O10,"")</f>
-        <v>-0.362116386110812</v>
+        <v>-0.36211634010729</v>
       </c>
       <c r="Q10" s="27" t="n">
         <f aca="false">IF(O10&gt;0,TDIST(ABS(P10),MIN(N27,N28)-1,2),"")</f>
-        <v>0.721481483979334</v>
+        <v>0.721481517766773</v>
       </c>
       <c r="R10" s="26" t="n">
         <v>-0.159163024562706</v>
@@ -8440,18 +8440,18 @@
         <v>0.915408975750982</v>
       </c>
       <c r="AD10" s="26" t="n">
-        <v>0.0176834769926367</v>
+        <v>0.0176834769928242</v>
       </c>
       <c r="AE10" s="26" t="n">
-        <v>0.178705604928376</v>
+        <v>0.17870561604616</v>
       </c>
       <c r="AF10" s="27" t="n">
         <f aca="false">IF(AE10&gt;0,AD10/AE10,"")</f>
-        <v>0.0989531190122665</v>
+        <v>0.0989531128571613</v>
       </c>
       <c r="AG10" s="27" t="n">
         <f aca="false">IF(AE10&gt;0,TDIST(ABS(AF10),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.92226917327103</v>
+        <v>0.922269178089429</v>
       </c>
       <c r="AH10" s="26" t="n">
         <v>-0.0434311694518283</v>
@@ -8496,18 +8496,18 @@
         <v>0.145575165147043</v>
       </c>
       <c r="AT10" s="26" t="n">
-        <v>-0.0913056549111026</v>
+        <v>-0.0913056549112335</v>
       </c>
       <c r="AU10" s="26" t="n">
-        <v>0.0556320006469363</v>
+        <v>0.0556319996183538</v>
       </c>
       <c r="AV10" s="27" t="n">
         <f aca="false">IF(AU10&gt;0,AT10/AU10,"")</f>
-        <v>-1.64124341834417</v>
+        <v>-1.64124344869154</v>
       </c>
       <c r="AW10" s="27" t="n">
         <f aca="false">IF(AU10&gt;0,TDIST(ABS(AV10),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.118103461259895</v>
+        <v>0.118103454911517</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8557,18 +8557,18 @@
         <v>0.271135280691244</v>
       </c>
       <c r="N11" s="26" t="n">
-        <v>-0.0786064517821817</v>
+        <v>-0.0786064517821275</v>
       </c>
       <c r="O11" s="26" t="n">
-        <v>0.0871212332954775</v>
+        <v>0.087121224515872</v>
       </c>
       <c r="P11" s="27" t="n">
         <f aca="false">IF(O11&gt;0,N11/O11,"")</f>
-        <v>-0.902265140296886</v>
+        <v>-0.902265231221661</v>
       </c>
       <c r="Q11" s="27" t="n">
         <f aca="false">IF(O11&gt;0,TDIST(ABS(P11),MIN(N27,N28)-1,2),"")</f>
-        <v>0.378831630165971</v>
+        <v>0.378831583166452</v>
       </c>
       <c r="R11" s="26" t="n">
         <v>-0.184360237730575</v>
@@ -8613,18 +8613,18 @@
         <v>0.783368415551846</v>
       </c>
       <c r="AD11" s="26" t="n">
-        <v>-0.0182543303453004</v>
+        <v>-0.0182543303450959</v>
       </c>
       <c r="AE11" s="26" t="n">
-        <v>0.168880151548657</v>
+        <v>0.168880162210197</v>
       </c>
       <c r="AF11" s="27" t="n">
         <f aca="false">IF(AE11&gt;0,AD11/AE11,"")</f>
-        <v>-0.108090442706886</v>
+        <v>-0.108090435881839</v>
       </c>
       <c r="AG11" s="27" t="n">
         <f aca="false">IF(AE11&gt;0,TDIST(ABS(AF11),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.915119716350208</v>
+        <v>0.915119721687725</v>
       </c>
       <c r="AH11" s="26" t="n">
         <v>-0.0324362470589291</v>
@@ -8669,18 +8669,18 @@
         <v>0.163073634181121</v>
       </c>
       <c r="AT11" s="26" t="n">
-        <v>-0.0869940324943472</v>
+        <v>-0.08699403249446</v>
       </c>
       <c r="AU11" s="26" t="n">
-        <v>0.0547187584925668</v>
+        <v>0.0547187569236586</v>
       </c>
       <c r="AV11" s="27" t="n">
         <f aca="false">IF(AU11&gt;0,AT11/AU11,"")</f>
-        <v>-1.58983929626555</v>
+        <v>-1.58983934185184</v>
       </c>
       <c r="AW11" s="27" t="n">
         <f aca="false">IF(AU11&gt;0,TDIST(ABS(AV11),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.129280724231395</v>
+        <v>0.129280713936456</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8730,18 +8730,18 @@
         <v>0.645675626469537</v>
       </c>
       <c r="N12" s="26" t="n">
-        <v>0.0109308959680605</v>
+        <v>0.0109308959681149</v>
       </c>
       <c r="O12" s="26" t="n">
-        <v>0.0941232546224913</v>
+        <v>0.0941232634532179</v>
       </c>
       <c r="P12" s="27" t="n">
         <f aca="false">IF(O12&gt;0,N12/O12,"")</f>
-        <v>0.116133850363568</v>
+        <v>0.116133839468368</v>
       </c>
       <c r="Q12" s="27" t="n">
         <f aca="false">IF(O12&gt;0,TDIST(ABS(P12),MIN(N27,N28)-1,2),"")</f>
-        <v>0.908832329671587</v>
+        <v>0.908832338184063</v>
       </c>
       <c r="R12" s="26" t="n">
         <v>-0.157671288557826</v>
@@ -8786,18 +8786,18 @@
         <v>0.900591747543548</v>
       </c>
       <c r="AD12" s="26" t="n">
-        <v>0.029712608230623</v>
+        <v>0.0297126082308318</v>
       </c>
       <c r="AE12" s="26" t="n">
-        <v>0.17402428857588</v>
+        <v>0.174024298418071</v>
       </c>
       <c r="AF12" s="27" t="n">
         <f aca="false">IF(AE12&gt;0,AD12/AE12,"")</f>
-        <v>0.170738282993568</v>
+        <v>0.170738273338422</v>
       </c>
       <c r="AG12" s="27" t="n">
         <f aca="false">IF(AE12&gt;0,TDIST(ABS(AF12),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.866334124157115</v>
+        <v>0.866334131638698</v>
       </c>
       <c r="AH12" s="26" t="n">
         <v>-0.034079724334971</v>
@@ -8842,18 +8842,18 @@
         <v>0.274769729770188</v>
       </c>
       <c r="AT12" s="26" t="n">
-        <v>-0.0646599021529623</v>
+        <v>-0.064659902153086</v>
       </c>
       <c r="AU12" s="26" t="n">
-        <v>0.0559097921130442</v>
+        <v>0.0559097900219613</v>
       </c>
       <c r="AV12" s="27" t="n">
         <f aca="false">IF(AU12&gt;0,AT12/AU12,"")</f>
-        <v>-1.15650407038227</v>
+        <v>-1.15650411363891</v>
       </c>
       <c r="AW12" s="27" t="n">
         <f aca="false">IF(AU12&gt;0,TDIST(ABS(AV12),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.26259408961956</v>
+        <v>0.262594072390983</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8903,18 +8903,18 @@
         <v>0.219020727999073</v>
       </c>
       <c r="N13" s="26" t="n">
-        <v>-0.0827138053070119</v>
+        <v>-0.0827138053069679</v>
       </c>
       <c r="O13" s="26" t="n">
-        <v>0.0740611260315613</v>
+        <v>0.0740611298118905</v>
       </c>
       <c r="P13" s="27" t="n">
         <f aca="false">IF(O13&gt;0,N13/O13,"")</f>
-        <v>-1.11683159221429</v>
+        <v>-1.11683153520686</v>
       </c>
       <c r="Q13" s="27" t="n">
         <f aca="false">IF(O13&gt;0,TDIST(ABS(P13),MIN(N27,N28)-1,2),"")</f>
-        <v>0.278753070315525</v>
+        <v>0.278753094051967</v>
       </c>
       <c r="R13" s="26" t="n">
         <v>-0.161413608888514</v>
@@ -8959,18 +8959,18 @@
         <v>0.970175883654116</v>
       </c>
       <c r="AD13" s="26" t="n">
-        <v>0.0118794834565776</v>
+        <v>0.0118794834567563</v>
       </c>
       <c r="AE13" s="26" t="n">
-        <v>0.170458793619823</v>
+        <v>0.170458804065296</v>
       </c>
       <c r="AF13" s="27" t="n">
         <f aca="false">IF(AE13&gt;0,AD13/AE13,"")</f>
-        <v>0.0696912327273218</v>
+        <v>0.0696912284577905</v>
       </c>
       <c r="AG13" s="27" t="n">
         <f aca="false">IF(AE13&gt;0,TDIST(ABS(AF13),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.945207829325238</v>
+        <v>0.945207832676266</v>
       </c>
       <c r="AH13" s="26" t="n">
         <v>-0.0218074512215736</v>
@@ -9015,18 +9015,18 @@
         <v>0.25823585510627</v>
       </c>
       <c r="AT13" s="26" t="n">
-        <v>-0.0690155442336617</v>
+        <v>-0.069015544233792</v>
       </c>
       <c r="AU13" s="26" t="n">
-        <v>0.0550184521037421</v>
+        <v>0.0550184506014438</v>
       </c>
       <c r="AV13" s="27" t="n">
         <f aca="false">IF(AU13&gt;0,AT13/AU13,"")</f>
-        <v>-1.25440723238682</v>
+        <v>-1.25440726664122</v>
       </c>
       <c r="AW13" s="27" t="n">
         <f aca="false">IF(AU13&gt;0,TDIST(ABS(AV13),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.225739268492852</v>
+        <v>0.225739256334969</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9076,18 +9076,18 @@
         <v>0.195534041346399</v>
       </c>
       <c r="N14" s="26" t="n">
-        <v>-0.0758237403895146</v>
+        <v>-0.0758237403894553</v>
       </c>
       <c r="O14" s="26" t="n">
-        <v>0.0862535459612432</v>
+        <v>0.0862535497230522</v>
       </c>
       <c r="P14" s="27" t="n">
         <f aca="false">IF(O14&gt;0,N14/O14,"")</f>
-        <v>-0.879079689356597</v>
+        <v>-0.87907965101627</v>
       </c>
       <c r="Q14" s="27" t="n">
         <f aca="false">IF(O14&gt;0,TDIST(ABS(P14),MIN(N27,N28)-1,2),"")</f>
-        <v>0.390942801651592</v>
+        <v>0.39094282188803</v>
       </c>
       <c r="R14" s="26" t="n">
         <v>-0.178658024977276</v>
@@ -9132,18 +9132,18 @@
         <v>0.896380032530518</v>
       </c>
       <c r="AD14" s="26" t="n">
-        <v>0.0337756347618206</v>
+        <v>0.0337756347620375</v>
       </c>
       <c r="AE14" s="26" t="n">
-        <v>0.180732976246689</v>
+        <v>0.180732992604367</v>
       </c>
       <c r="AF14" s="27" t="n">
         <f aca="false">IF(AE14&gt;0,AD14/AE14,"")</f>
-        <v>0.18688141734422</v>
+        <v>0.186881400431265</v>
       </c>
       <c r="AG14" s="27" t="n">
         <f aca="false">IF(AE14&gt;0,TDIST(ABS(AF14),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.853843840265806</v>
+        <v>0.853843853331525</v>
       </c>
       <c r="AH14" s="26" t="n">
         <v>-0.0339578513977617</v>
@@ -9188,18 +9188,18 @@
         <v>0.222552025486122</v>
       </c>
       <c r="AT14" s="26" t="n">
-        <v>-0.0731888883192778</v>
+        <v>-0.0731888883194041</v>
       </c>
       <c r="AU14" s="26" t="n">
-        <v>0.0551493075815952</v>
+        <v>0.0551493060504304</v>
       </c>
       <c r="AV14" s="27" t="n">
         <f aca="false">IF(AU14&gt;0,AT14/AU14,"")</f>
-        <v>-1.3271043922173</v>
+        <v>-1.3271044290653</v>
       </c>
       <c r="AW14" s="27" t="n">
         <f aca="false">IF(AU14&gt;0,TDIST(ABS(AV14),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.201063167850877</v>
+        <v>0.201063155905873</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9249,18 +9249,18 @@
         <v>0.162102167594176</v>
       </c>
       <c r="N15" s="26" t="n">
-        <v>-0.123404989476307</v>
+        <v>-0.123404989476236</v>
       </c>
       <c r="O15" s="26" t="n">
-        <v>0.0983379140108944</v>
+        <v>0.0983379213104224</v>
       </c>
       <c r="P15" s="27" t="n">
         <f aca="false">IF(O15&gt;0,N15/O15,"")</f>
-        <v>-1.25490753711366</v>
+        <v>-1.25490744396238</v>
       </c>
       <c r="Q15" s="27" t="n">
         <f aca="false">IF(O15&gt;0,TDIST(ABS(P15),MIN(N27,N28)-1,2),"")</f>
-        <v>0.225561749905134</v>
+        <v>0.225561782947089</v>
       </c>
       <c r="R15" s="26" t="n">
         <v>-0.197812493908102</v>
@@ -9305,18 +9305,18 @@
         <v>0.862606334604382</v>
       </c>
       <c r="AD15" s="26" t="n">
-        <v>0.00333965441158022</v>
+        <v>0.00333965441181926</v>
       </c>
       <c r="AE15" s="26" t="n">
-        <v>0.173188236648948</v>
+        <v>0.173188256185137</v>
       </c>
       <c r="AF15" s="27" t="n">
         <f aca="false">IF(AE15&gt;0,AD15/AE15,"")</f>
-        <v>0.0192833790342799</v>
+        <v>0.0192833768604332</v>
       </c>
       <c r="AG15" s="27" t="n">
         <f aca="false">IF(AE15&gt;0,TDIST(ABS(AF15),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.984827190216257</v>
+        <v>0.984827191926452</v>
       </c>
       <c r="AH15" s="26" t="n">
         <v>-0.0320791887764176</v>
@@ -9361,18 +9361,18 @@
         <v>0.175347306906619</v>
       </c>
       <c r="AT15" s="26" t="n">
-        <v>-0.0825527442173372</v>
+        <v>-0.0825527442174579</v>
       </c>
       <c r="AU15" s="26" t="n">
-        <v>0.0541670437764627</v>
+        <v>0.0541670423530397</v>
       </c>
       <c r="AV15" s="27" t="n">
         <f aca="false">IF(AU15&gt;0,AT15/AU15,"")</f>
-        <v>-1.52404005206592</v>
+        <v>-1.52404009211748</v>
       </c>
       <c r="AW15" s="27" t="n">
         <f aca="false">IF(AU15&gt;0,TDIST(ABS(AV15),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.144875522314131</v>
+        <v>0.14487551236474</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9422,18 +9422,18 @@
         <v>0.549204381894683</v>
       </c>
       <c r="N16" s="26" t="n">
-        <v>-0.0461957598888445</v>
+        <v>-0.0461957598887847</v>
       </c>
       <c r="O16" s="26" t="n">
-        <v>0.113729266084523</v>
+        <v>0.113729252783398</v>
       </c>
       <c r="P16" s="27" t="n">
         <f aca="false">IF(O16&gt;0,N16/O16,"")</f>
-        <v>-0.406190609324005</v>
+        <v>-0.406190656829218</v>
       </c>
       <c r="Q16" s="27" t="n">
         <f aca="false">IF(O16&gt;0,TDIST(ABS(P16),MIN(N27,N28)-1,2),"")</f>
-        <v>0.689390888049788</v>
+        <v>0.68939085377245</v>
       </c>
       <c r="R16" s="26" t="n">
         <v>-0.125685164309483</v>
@@ -9478,18 +9478,18 @@
         <v>0.853989365834896</v>
       </c>
       <c r="AD16" s="26" t="n">
-        <v>0.0634489420482868</v>
+        <v>0.0634489420485265</v>
       </c>
       <c r="AE16" s="26" t="n">
-        <v>0.186944390685094</v>
+        <v>0.186944407118613</v>
       </c>
       <c r="AF16" s="27" t="n">
         <f aca="false">IF(AE16&gt;0,AD16/AE16,"")</f>
-        <v>0.339400084783318</v>
+        <v>0.339400054949327</v>
       </c>
       <c r="AG16" s="27" t="n">
         <f aca="false">IF(AE16&gt;0,TDIST(ABS(AF16),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.738236170882535</v>
+        <v>0.738236192978012</v>
       </c>
       <c r="AH16" s="26" t="n">
         <v>-0.0363159348805042</v>
@@ -9534,18 +9534,18 @@
         <v>0.19396341621592</v>
       </c>
       <c r="AT16" s="26" t="n">
-        <v>-0.0797540683619493</v>
+        <v>-0.0797540683620755</v>
       </c>
       <c r="AU16" s="26" t="n">
-        <v>0.0554049470335655</v>
+        <v>0.0554049452905511</v>
       </c>
       <c r="AV16" s="27" t="n">
         <f aca="false">IF(AU16&gt;0,AT16/AU16,"")</f>
-        <v>-1.43947558173158</v>
+        <v>-1.43947562701911</v>
       </c>
       <c r="AW16" s="27" t="n">
         <f aca="false">IF(AU16&gt;0,TDIST(ABS(AV16),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.167180594748092</v>
+        <v>0.16718058209056</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9670,18 +9670,18 @@
         <v>0.218273654085262</v>
       </c>
       <c r="N18" s="26" t="n">
-        <v>0.916112060092399</v>
+        <v>0.9161120600929</v>
       </c>
       <c r="O18" s="26" t="n">
-        <v>0.669547617873632</v>
+        <v>0.66954779166628</v>
       </c>
       <c r="P18" s="27" t="n">
         <f aca="false">IF(O18&gt;0,N18/O18,"")</f>
-        <v>1.3682552751092</v>
+        <v>1.36825491995576</v>
       </c>
       <c r="Q18" s="27" t="n">
         <f aca="false">IF(O18&gt;0,TDIST(ABS(P18),MIN(N27,N28)-1,2),"")</f>
-        <v>0.188070321457473</v>
+        <v>0.188070430625583</v>
       </c>
       <c r="V18" s="26" t="n">
         <v>-1.20970864400307</v>
@@ -9712,18 +9712,18 @@
         <v>0.822940375760089</v>
       </c>
       <c r="AD18" s="26" t="n">
-        <v>0.211101290447338</v>
+        <v>0.211101290449027</v>
       </c>
       <c r="AE18" s="26" t="n">
-        <v>0.68883936179849</v>
+        <v>0.688839603917236</v>
       </c>
       <c r="AF18" s="27" t="n">
         <f aca="false">IF(AE18&gt;0,AD18/AE18,"")</f>
-        <v>0.306459389742441</v>
+        <v>0.306459282028143</v>
       </c>
       <c r="AG18" s="27" t="n">
         <f aca="false">IF(AE18&gt;0,TDIST(ABS(AF18),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.76277150381195</v>
+        <v>0.76277158448226</v>
       </c>
       <c r="AL18" s="26" t="n">
         <v>0.000657320869398719</v>
@@ -9754,18 +9754,18 @@
         <v>0.0920547807372332</v>
       </c>
       <c r="AT18" s="26" t="n">
-        <v>-0.154935049159671</v>
+        <v>-0.154935049161262</v>
       </c>
       <c r="AU18" s="26" t="n">
-        <v>0.103762778880472</v>
+        <v>0.103762837057385</v>
       </c>
       <c r="AV18" s="27" t="n">
         <f aca="false">IF(AU18&gt;0,AT18/AU18,"")</f>
-        <v>-1.49316595826858</v>
+        <v>-1.49316512110764</v>
       </c>
       <c r="AW18" s="27" t="n">
         <f aca="false">IF(AU18&gt;0,TDIST(ABS(AV18),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.152715383181071</v>
+        <v>0.152715600421818</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9801,18 +9801,18 @@
         <v>0.919415775750922</v>
       </c>
       <c r="N19" s="26" t="n">
-        <v>-0.036556546968862</v>
+        <v>-0.0365565469689395</v>
       </c>
       <c r="O19" s="26" t="n">
-        <v>0.128747992961838</v>
+        <v>0.128747997801159</v>
       </c>
       <c r="P19" s="27" t="n">
         <f aca="false">IF(O19&gt;0,N19/O19,"")</f>
-        <v>-0.283938771610193</v>
+        <v>-0.283938760938234</v>
       </c>
       <c r="Q19" s="27" t="n">
         <f aca="false">IF(O19&gt;0,TDIST(ABS(P19),MIN(N27,N28)-1,2),"")</f>
-        <v>0.77969761165244</v>
+        <v>0.779697619700987</v>
       </c>
       <c r="V19" s="26" t="n">
         <v>-0.0115424232164245</v>
@@ -9843,18 +9843,18 @@
         <v>0.529864445684847</v>
       </c>
       <c r="AD19" s="26" t="n">
-        <v>-0.192928025021406</v>
+        <v>-0.192928025021655</v>
       </c>
       <c r="AE19" s="26" t="n">
-        <v>0.131562080853572</v>
+        <v>0.131562048752238</v>
       </c>
       <c r="AF19" s="27" t="n">
         <f aca="false">IF(AE19&gt;0,AD19/AE19,"")</f>
-        <v>-1.46644096665007</v>
+        <v>-1.46644132446572</v>
       </c>
       <c r="AG19" s="27" t="n">
         <f aca="false">IF(AE19&gt;0,TDIST(ABS(AF19),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.159781410357885</v>
+        <v>0.159781313985108</v>
       </c>
       <c r="AL19" s="26" t="n">
         <v>-0.0148866300368887</v>
@@ -9885,18 +9885,18 @@
         <v>0.134842824678975</v>
       </c>
       <c r="AT19" s="26" t="n">
-        <v>0.0135682955824442</v>
+        <v>0.0135682955825505</v>
       </c>
       <c r="AU19" s="26" t="n">
-        <v>0.00997984813497247</v>
+        <v>0.00997984614003043</v>
       </c>
       <c r="AV19" s="27" t="n">
         <f aca="false">IF(AU19&gt;0,AT19/AU19,"")</f>
-        <v>1.35956934403608</v>
+        <v>1.35956961582066</v>
       </c>
       <c r="AW19" s="27" t="n">
         <f aca="false">IF(AU19&gt;0,TDIST(ABS(AV19),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.190755428229536</v>
+        <v>0.190755343735404</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9932,18 +9932,18 @@
         <v>0.825682762760703</v>
       </c>
       <c r="N20" s="26" t="n">
-        <v>0.00411152095119167</v>
+        <v>0.00411152095117649</v>
       </c>
       <c r="O20" s="26" t="n">
-        <v>0.157021531202805</v>
+        <v>0.157021551197996</v>
       </c>
       <c r="P20" s="27" t="n">
         <f aca="false">IF(O20&gt;0,N20/O20,"")</f>
-        <v>0.0261844405649143</v>
+        <v>0.0261844372304798</v>
       </c>
       <c r="Q20" s="27" t="n">
         <f aca="false">IF(O20&gt;0,TDIST(ABS(P20),MIN(N27,N28)-1,2),"")</f>
-        <v>0.979398340567554</v>
+        <v>0.979398343190407</v>
       </c>
       <c r="V20" s="26" t="n">
         <v>0.102290343172575</v>
@@ -9974,18 +9974,18 @@
         <v>0.514674983751795</v>
       </c>
       <c r="AD20" s="26" t="n">
-        <v>0.107305976151842</v>
+        <v>0.10730597615155</v>
       </c>
       <c r="AE20" s="26" t="n">
-        <v>0.210124306687761</v>
+        <v>0.210124279872008</v>
       </c>
       <c r="AF20" s="27" t="n">
         <f aca="false">IF(AE20&gt;0,AD20/AE20,"")</f>
-        <v>0.510678549489733</v>
+        <v>0.510678614660392</v>
       </c>
       <c r="AG20" s="27" t="n">
         <f aca="false">IF(AE20&gt;0,TDIST(ABS(AF20),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.615782238688105</v>
+        <v>0.615782193956367</v>
       </c>
       <c r="AL20" s="26" t="n">
         <v>-0.0561646633488208</v>
@@ -10016,18 +10016,18 @@
         <v>0.189347131150784</v>
       </c>
       <c r="AT20" s="26" t="n">
-        <v>-0.0674280072932556</v>
+        <v>-0.0674280072933353</v>
       </c>
       <c r="AU20" s="26" t="n">
-        <v>0.0511512392360329</v>
+        <v>0.0511512406609408</v>
       </c>
       <c r="AV20" s="27" t="n">
         <f aca="false">IF(AU20&gt;0,AT20/AU20,"")</f>
-        <v>-1.31820867490844</v>
+        <v>-1.31820863818897</v>
       </c>
       <c r="AW20" s="27" t="n">
         <f aca="false">IF(AU20&gt;0,TDIST(ABS(AV20),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.203963287346734</v>
+        <v>0.203963299385575</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10063,18 +10063,18 @@
         <v>0.327826327627622</v>
       </c>
       <c r="N21" s="26" t="n">
-        <v>0.28856215094249</v>
+        <v>0.288562150942612</v>
       </c>
       <c r="O21" s="26" t="n">
-        <v>0.239714292238323</v>
+        <v>0.239714276931182</v>
       </c>
       <c r="P21" s="27" t="n">
         <f aca="false">IF(O21&gt;0,N21/O21,"")</f>
-        <v>1.20377532873844</v>
+        <v>1.20377540560696</v>
       </c>
       <c r="Q21" s="27" t="n">
         <f aca="false">IF(O21&gt;0,TDIST(ABS(P21),MIN(N27,N28)-1,2),"")</f>
-        <v>0.244268945399072</v>
+        <v>0.244268916411721</v>
       </c>
       <c r="V21" s="26" t="n">
         <v>-0.154069789120528</v>
@@ -10105,18 +10105,18 @@
         <v>0.612949024871307</v>
       </c>
       <c r="AD21" s="26" t="n">
-        <v>-0.0165841587906105</v>
+        <v>-0.0165841587901762</v>
       </c>
       <c r="AE21" s="26" t="n">
-        <v>0.211298211443597</v>
+        <v>0.211298198134876</v>
       </c>
       <c r="AF21" s="27" t="n">
         <f aca="false">IF(AE21&gt;0,AD21/AE21,"")</f>
-        <v>-0.0784869813961364</v>
+        <v>-0.0784869863376223</v>
       </c>
       <c r="AG21" s="27" t="n">
         <f aca="false">IF(AE21&gt;0,TDIST(ABS(AF21),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.93830662896342</v>
+        <v>0.938306625087648</v>
       </c>
       <c r="AL21" s="26" t="n">
         <v>0.0326969620171097</v>
@@ -10147,18 +10147,18 @@
         <v>0.135787413205493</v>
       </c>
       <c r="AT21" s="26" t="n">
-        <v>-0.0586225463289042</v>
+        <v>-0.0586225463287142</v>
       </c>
       <c r="AU21" s="26" t="n">
-        <v>0.035888646339194</v>
+        <v>0.0358886348798194</v>
       </c>
       <c r="AV21" s="27" t="n">
         <f aca="false">IF(AU21&gt;0,AT21/AU21,"")</f>
-        <v>-1.63345660281654</v>
+        <v>-1.63345712438002</v>
       </c>
       <c r="AW21" s="27" t="n">
         <f aca="false">IF(AU21&gt;0,TDIST(ABS(AV21),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.119741971172003</v>
+        <v>0.119741860780472</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10194,18 +10194,18 @@
         <v>0.763025335695412</v>
       </c>
       <c r="N22" s="26" t="n">
-        <v>-0.186903281953439</v>
+        <v>-0.186903281951916</v>
       </c>
       <c r="O22" s="26" t="n">
-        <v>0.986290901623803</v>
+        <v>0.98629075151137</v>
       </c>
       <c r="P22" s="27" t="n">
         <f aca="false">IF(O22&gt;0,N22/O22,"")</f>
-        <v>-0.189501172165055</v>
+        <v>-0.189501201005393</v>
       </c>
       <c r="Q22" s="27" t="n">
         <f aca="false">IF(O22&gt;0,TDIST(ABS(P22),MIN(N27,N28)-1,2),"")</f>
-        <v>0.85182053199935</v>
+        <v>0.851820509730958</v>
       </c>
       <c r="V22" s="26" t="n">
         <v>0.314236553362949</v>
@@ -10236,18 +10236,18 @@
         <v>0.960143749884991</v>
       </c>
       <c r="AD22" s="26" t="n">
-        <v>0.540754698469919</v>
+        <v>0.540754698476038</v>
       </c>
       <c r="AE22" s="26" t="n">
-        <v>0.753742850699821</v>
+        <v>0.753743317861591</v>
       </c>
       <c r="AF22" s="27" t="n">
         <f aca="false">IF(AE22&gt;0,AD22/AE22,"")</f>
-        <v>0.717425973550328</v>
+        <v>0.717425528905764</v>
       </c>
       <c r="AG22" s="27" t="n">
         <f aca="false">IF(AE22&gt;0,TDIST(ABS(AF22),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.482318690730375</v>
+        <v>0.482318958403444</v>
       </c>
       <c r="AL22" s="26" t="n">
         <v>0.00246903924119752</v>
@@ -10278,18 +10278,18 @@
         <v>0.00232058632969922</v>
       </c>
       <c r="AT22" s="26" t="n">
-        <v>-0.255506195426355</v>
+        <v>-0.255506195424912</v>
       </c>
       <c r="AU22" s="26" t="n">
-        <v>0.0793685541710431</v>
+        <v>0.0793685224677337</v>
       </c>
       <c r="AV22" s="27" t="n">
         <f aca="false">IF(AU22&gt;0,AT22/AU22,"")</f>
-        <v>-3.21923711594552</v>
+        <v>-3.21923840183348</v>
       </c>
       <c r="AW22" s="27" t="n">
         <f aca="false">IF(AU22&gt;0,TDIST(ABS(AV22),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.00475692079584615</v>
+        <v>0.00475690733767288</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10325,18 +10325,18 @@
         <v>0.967385354514503</v>
       </c>
       <c r="N23" s="26" t="n">
-        <v>-0.466461783464562</v>
+        <v>-0.466461783466271</v>
       </c>
       <c r="O23" s="26" t="n">
-        <v>1.65177888349339</v>
+        <v>1.65177885922458</v>
       </c>
       <c r="P23" s="27" t="n">
         <f aca="false">IF(O23&gt;0,N23/O23,"")</f>
-        <v>-0.28239965295962</v>
+        <v>-0.28239965710982</v>
       </c>
       <c r="Q23" s="27" t="n">
         <f aca="false">IF(O23&gt;0,TDIST(ABS(P23),MIN(N27,N28)-1,2),"")</f>
-        <v>0.780858645615495</v>
+        <v>0.78085864248408</v>
       </c>
       <c r="V23" s="26" t="n">
         <v>-0.0418925589087689</v>
@@ -10367,18 +10367,18 @@
         <v>0.81446146784386</v>
       </c>
       <c r="AD23" s="26" t="n">
-        <v>-0.322203311697373</v>
+        <v>-0.322203311698105</v>
       </c>
       <c r="AE23" s="26" t="n">
-        <v>1.32734432207094</v>
+        <v>1.32734499211575</v>
       </c>
       <c r="AF23" s="27" t="n">
         <f aca="false">IF(AE23&gt;0,AD23/AE23,"")</f>
-        <v>-0.242742825911718</v>
+        <v>-0.242742703375497</v>
       </c>
       <c r="AG23" s="27" t="n">
         <f aca="false">IF(AE23&gt;0,TDIST(ABS(AF23),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.810949136049983</v>
+        <v>0.810949229524189</v>
       </c>
       <c r="AL23" s="26" t="n">
         <v>-0.0767536935021354</v>
@@ -10409,18 +10409,18 @@
         <v>0.598948466684306</v>
       </c>
       <c r="AT23" s="26" t="n">
-        <v>-0.118423192725048</v>
+        <v>-0.118423192725193</v>
       </c>
       <c r="AU23" s="26" t="n">
-        <v>0.134514794829928</v>
+        <v>0.134514797999034</v>
       </c>
       <c r="AV23" s="27" t="n">
         <f aca="false">IF(AU23&gt;0,AT23/AU23,"")</f>
-        <v>-0.880372994470794</v>
+        <v>-0.880372973730692</v>
       </c>
       <c r="AW23" s="27" t="n">
         <f aca="false">IF(AU23&gt;0,TDIST(ABS(AV23),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.390260574074749</v>
+        <v>0.390260585009001</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10470,18 +10470,18 @@
         <v>0.320694339145249</v>
       </c>
       <c r="N24" s="26" t="n">
-        <v>-0.282303553782618</v>
+        <v>-0.282303553782655</v>
       </c>
       <c r="O24" s="26" t="n">
-        <v>0.233335247759787</v>
+        <v>0.233335255365373</v>
       </c>
       <c r="P24" s="27" t="n">
         <f aca="false">IF(O24&gt;0,N24/O24,"")</f>
-        <v>-1.20986244681405</v>
+        <v>-1.20986240737862</v>
       </c>
       <c r="Q24" s="27" t="n">
         <f aca="false">IF(O24&gt;0,TDIST(ABS(P24),MIN(N27,N28)-1,2),"")</f>
-        <v>0.241981682651842</v>
+        <v>0.241981697416763</v>
       </c>
       <c r="R24" s="26" t="n">
         <v>-0.155888707699309</v>
@@ -10526,18 +10526,18 @@
         <v>0.190500893906074</v>
       </c>
       <c r="AD24" s="26" t="n">
-        <v>-0.43635533666787</v>
+        <v>-0.436355336668285</v>
       </c>
       <c r="AE24" s="26" t="n">
-        <v>0.248107304107821</v>
+        <v>0.248107268976187</v>
       </c>
       <c r="AF24" s="27" t="n">
         <f aca="false">IF(AE24&gt;0,AD24/AE24,"")</f>
-        <v>-1.7587363589999</v>
+        <v>-1.75873660803612</v>
       </c>
       <c r="AG24" s="27" t="n">
         <f aca="false">IF(AE24&gt;0,TDIST(ABS(AF24),MIN(AD27,AD28)-1,2),"")</f>
-        <v>0.0956110552579578</v>
+        <v>0.0956110118151261</v>
       </c>
       <c r="AH24" s="26" t="n">
         <v>0.00208687491540036</v>
@@ -10582,18 +10582,18 @@
         <v>0.849413111405078</v>
       </c>
       <c r="AT24" s="26" t="n">
-        <v>0.00867134554664069</v>
+        <v>0.00867134554684633</v>
       </c>
       <c r="AU24" s="26" t="n">
-        <v>0.0379095017955387</v>
+        <v>0.0379095014949195</v>
       </c>
       <c r="AV24" s="27" t="n">
         <f aca="false">IF(AU24&gt;0,AT24/AU24,"")</f>
-        <v>0.228738050777052</v>
+        <v>0.228738052596351</v>
       </c>
       <c r="AW24" s="27" t="n">
         <f aca="false">IF(AU24&gt;0,TDIST(ABS(AV24),MIN(AT27,AT28)-1,2),"")</f>
-        <v>0.821651149356285</v>
+        <v>0.821651147963641</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10733,7 +10733,7 @@
         <v>0.0805095842434804</v>
       </c>
       <c r="N29" s="20" t="n">
-        <v>0.0952588261959438</v>
+        <v>0.095258826195944</v>
       </c>
       <c r="R29" s="20" t="n">
         <v>0.118578094817697</v>
@@ -10745,7 +10745,7 @@
         <v>0.0207914424340943</v>
       </c>
       <c r="AD29" s="20" t="n">
-        <v>0.12390479939966</v>
+        <v>0.123904799399671</v>
       </c>
       <c r="AH29" s="20" t="n">
         <v>0.342677598096958</v>
@@ -10757,7 +10757,7 @@
         <v>0.661655111871864</v>
       </c>
       <c r="AT29" s="20" t="n">
-        <v>0.670564522582896</v>
+        <v>0.67056452258284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>